<commit_message>
added tables to the lana_dog_walking schema updated the Excel worksheet to be more visually appealing
</commit_message>
<xml_diff>
--- a/Mrapshtija_Ex3A_tables.xlsx
+++ b/Mrapshtija_Ex3A_tables.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arditamrapshtija\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D313534-E597-41FE-9404-6FF05386A300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E885FC0F-4576-4E86-98B8-833EE11FC5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{29F24C90-C5E6-43D8-A5C9-943B7BC280D5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Owner" sheetId="1" r:id="rId1"/>
+    <sheet name="Dog" sheetId="2" r:id="rId2"/>
+    <sheet name="Walk" sheetId="3" r:id="rId3"/>
+    <sheet name="Payment" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,9 +44,68 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="19" uniqueCount="18">
+  <si>
+    <t>owner_name</t>
+  </si>
+  <si>
+    <t>phone_number</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>owner_id (PK)</t>
+  </si>
+  <si>
+    <t>dog_id (PK)</t>
+  </si>
+  <si>
+    <t>dog_name</t>
+  </si>
+  <si>
+    <t>breed</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>owner_id (FK)</t>
+  </si>
+  <si>
+    <t>walk_date</t>
+  </si>
+  <si>
+    <t>walk_duration</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>walk_id (PK)</t>
+  </si>
+  <si>
+    <t>dog_id (FK)</t>
+  </si>
+  <si>
+    <t>payment_id(PK)</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>payment_method</t>
+  </si>
+  <si>
+    <t>date_serviced</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -51,13 +113,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -72,13 +159,296 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="19">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -89,6 +459,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B335E5B2-B7AD-4762-BF44-C42AA3E92FDB}" name="Table3" displayName="Table3" ref="A1:D6" totalsRowShown="0" headerRowDxfId="18">
+  <autoFilter ref="A1:D6" xr:uid="{B335E5B2-B7AD-4762-BF44-C42AA3E92FDB}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{80C424CD-BB3A-4298-8A33-4AB14830922C}" name="owner_id (PK)" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{868B76BA-5E64-4B57-B52D-01AE590DF59A}" name="owner_name"/>
+    <tableColumn id="3" xr3:uid="{AE0EA7D6-324F-4022-949D-B36D24E721B1}" name="phone_number"/>
+    <tableColumn id="4" xr3:uid="{4F399586-F23F-45A5-8233-15FA5DF37BD4}" name="email"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{139D2D28-EFCC-49C1-A53E-E235293ADC54}" name="Table4" displayName="Table4" ref="A1:E6" totalsRowShown="0" headerRowDxfId="14">
+  <autoFilter ref="A1:E6" xr:uid="{139D2D28-EFCC-49C1-A53E-E235293ADC54}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{C9C10A94-BBB3-43C0-968B-38EE22385182}" name="dog_id (PK)" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{C2714D09-162B-4C42-8B5D-7229997503D1}" name="owner_id (FK)" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{34445534-D457-4D7F-8C6A-4E28ED4FA7DC}" name="dog_name"/>
+    <tableColumn id="4" xr3:uid="{21D784F5-21C4-474F-9CF7-F7A6E1AA51BB}" name="breed"/>
+    <tableColumn id="5" xr3:uid="{8F63065B-72DA-4B93-80DB-A547E9CD3F3D}" name="age"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6C4E8387-2403-4929-A86F-6A75BFD444B5}" name="Table5" displayName="Table5" ref="A1:E6" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:E6" xr:uid="{6C4E8387-2403-4929-A86F-6A75BFD444B5}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{06E20231-D9AB-41BF-BEF3-7116BE749241}" name="walk_id (PK)" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{6500AF60-F9C5-41CD-A427-7C0FC3A4BFA7}" name="dog_id (FK)" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{933DB32B-8DA0-4A67-9221-9B8167AEB156}" name="walk_date" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{37A70DF2-1F30-43B3-A7C1-D69E5EB18474}" name="walk_duration" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{55C5F72B-9A3E-4203-9581-EA680786B0ED}" name="notes" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{443EBC68-654A-40F9-9C0D-814B574680F5}" name="Table6" displayName="Table6" ref="A1:E7" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:E7" xr:uid="{443EBC68-654A-40F9-9C0D-814B574680F5}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{7BC331FF-D9AF-4646-A8C9-A1CC322052CB}" name="payment_id(PK)" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{435F1D1D-4E2F-4B4A-8EE2-1A1D5882592A}" name="owner_id (FK)" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{540F89FC-A9E4-4B8D-8383-1F058B36C275}" name="amount" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{C99CE62D-56AA-4875-885E-270D551F0932}" name="payment_method" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{1FAD9FA5-F486-47DD-BAA1-6CA888E42A56}" name="date_serviced" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -408,9 +833,236 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87CA01F9-40B5-46BE-BE52-FFD169ED4555}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="4"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31BC9D7B-BD90-455D-9CF5-F52E79C3F8D6}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB45426-463C-4A45-B6CF-E0C9E34E5E52}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EBFFC7A-9C7A-4EF9-AAD2-CC05C51D2EE7}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="8"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated the Excel Workbook with the sample records inserted the sample records into the schema
</commit_message>
<xml_diff>
--- a/Mrapshtija_Ex3A_tables.xlsx
+++ b/Mrapshtija_Ex3A_tables.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arditamrapshtija\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E885FC0F-4576-4E86-98B8-833EE11FC5F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F326F65F-11B0-4C72-902E-C73E2D755FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{29F24C90-C5E6-43D8-A5C9-943B7BC280D5}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{29F24C90-C5E6-43D8-A5C9-943B7BC280D5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Owner" sheetId="1" r:id="rId1"/>
-    <sheet name="Dog" sheetId="2" r:id="rId2"/>
-    <sheet name="Walk" sheetId="3" r:id="rId3"/>
-    <sheet name="Payment" sheetId="4" r:id="rId4"/>
+    <sheet name="owner" sheetId="1" r:id="rId1"/>
+    <sheet name="dog" sheetId="2" r:id="rId2"/>
+    <sheet name="walk" sheetId="3" r:id="rId3"/>
+    <sheet name="payment" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="19" uniqueCount="18">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="96" uniqueCount="88">
   <si>
     <t>owner_name</t>
   </si>
@@ -56,12 +56,6 @@
     <t>email</t>
   </si>
   <si>
-    <t>owner_id (PK)</t>
-  </si>
-  <si>
-    <t>dog_id (PK)</t>
-  </si>
-  <si>
     <t>dog_name</t>
   </si>
   <si>
@@ -71,9 +65,6 @@
     <t>age</t>
   </si>
   <si>
-    <t>owner_id (FK)</t>
-  </si>
-  <si>
     <t>walk_date</t>
   </si>
   <si>
@@ -83,15 +74,6 @@
     <t>notes</t>
   </si>
   <si>
-    <t>walk_id (PK)</t>
-  </si>
-  <si>
-    <t>dog_id (FK)</t>
-  </si>
-  <si>
-    <t>payment_id(PK)</t>
-  </si>
-  <si>
     <t>amount</t>
   </si>
   <si>
@@ -99,13 +81,246 @@
   </si>
   <si>
     <t>date_serviced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">owner_id </t>
+  </si>
+  <si>
+    <t xml:space="preserve">dog_id </t>
+  </si>
+  <si>
+    <t xml:space="preserve">walk_id </t>
+  </si>
+  <si>
+    <t>payment_id</t>
+  </si>
+  <si>
+    <t>Maria Santos</t>
+  </si>
+  <si>
+    <t>555-123-4567</t>
+  </si>
+  <si>
+    <t>maria.santos@example.com</t>
+  </si>
+  <si>
+    <t>Biscuit</t>
+  </si>
+  <si>
+    <t>Golden Retriever</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very energetic. Walked around the park and met two other dogs. </t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>James Okafor</t>
+  </si>
+  <si>
+    <t>555-234-5678</t>
+  </si>
+  <si>
+    <t>james.okafor@example.com</t>
+  </si>
+  <si>
+    <t>Priya Patel</t>
+  </si>
+  <si>
+    <t>555-345-6789</t>
+  </si>
+  <si>
+    <t>priya.patel@example.com</t>
+  </si>
+  <si>
+    <t>Daniel Kim</t>
+  </si>
+  <si>
+    <t>555-456-7890</t>
+  </si>
+  <si>
+    <t>daniel.kim@example.com</t>
+  </si>
+  <si>
+    <t>Emily Johnson</t>
+  </si>
+  <si>
+    <t>555-567-8901</t>
+  </si>
+  <si>
+    <t>emily.johnson@example.com</t>
+  </si>
+  <si>
+    <t>Carlos Ramirez</t>
+  </si>
+  <si>
+    <t>555-678-9012</t>
+  </si>
+  <si>
+    <t>carlos.ramirez@example.com</t>
+  </si>
+  <si>
+    <t>Aisha Rahman</t>
+  </si>
+  <si>
+    <t>555-789-0123</t>
+  </si>
+  <si>
+    <t>aisha.rahman@example.com</t>
+  </si>
+  <si>
+    <t>Thomas Becker</t>
+  </si>
+  <si>
+    <t>555-890-1234</t>
+  </si>
+  <si>
+    <t>thomas.becker@example.com</t>
+  </si>
+  <si>
+    <t>Sofia Rossi</t>
+  </si>
+  <si>
+    <t>555-901-2345</t>
+  </si>
+  <si>
+    <t>sofia.rossi@example.com</t>
+  </si>
+  <si>
+    <t>Michael O'Brien</t>
+  </si>
+  <si>
+    <t>555-012-3456</t>
+  </si>
+  <si>
+    <t>michael.obrien@example.com</t>
+  </si>
+  <si>
+    <t>Hannah Lee</t>
+  </si>
+  <si>
+    <t>555-123-9876</t>
+  </si>
+  <si>
+    <t>hannah.lee@example.com</t>
+  </si>
+  <si>
+    <t>Luna</t>
+  </si>
+  <si>
+    <t>Labrador Retriever</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>German Shepherd</t>
+  </si>
+  <si>
+    <t>Bella</t>
+  </si>
+  <si>
+    <t>Beagle</t>
+  </si>
+  <si>
+    <t>Charlie</t>
+  </si>
+  <si>
+    <t>French Bulldog</t>
+  </si>
+  <si>
+    <t>Daisy</t>
+  </si>
+  <si>
+    <t>Poodle</t>
+  </si>
+  <si>
+    <t>Rocky</t>
+  </si>
+  <si>
+    <t>Boxer</t>
+  </si>
+  <si>
+    <t>Cooper</t>
+  </si>
+  <si>
+    <t>Border Collie</t>
+  </si>
+  <si>
+    <t>Milo</t>
+  </si>
+  <si>
+    <t>Dachshund</t>
+  </si>
+  <si>
+    <t>Teddy</t>
+  </si>
+  <si>
+    <t>Siberian Husky</t>
+  </si>
+  <si>
+    <t>Zoe</t>
+  </si>
+  <si>
+    <t>Corgi</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Venmo</t>
+  </si>
+  <si>
+    <t>Debit Card</t>
+  </si>
+  <si>
+    <t>PayPal</t>
+  </si>
+  <si>
+    <t>Zelle</t>
+  </si>
+  <si>
+    <t>Luna pulled on the leash at first but calmed down.</t>
+  </si>
+  <si>
+    <t>Long walk through the neighborhood. Max was well behaved.</t>
+  </si>
+  <si>
+    <t>Bella followed scents the whole walk.</t>
+  </si>
+  <si>
+    <t>Short walk due to warm weather. Gave water afterward.</t>
+  </si>
+  <si>
+    <t>Daisy enjoyed meeting other dogs at the park.</t>
+  </si>
+  <si>
+    <t>Rocky had lots of energy. Played fetch at the end.</t>
+  </si>
+  <si>
+    <t>Cooper did great with commands at the dog park.</t>
+  </si>
+  <si>
+    <t>Milo stopped often to sniff. No issues.</t>
+  </si>
+  <si>
+    <t>Teddy ran the trail loop and was tired afterward.</t>
+  </si>
+  <si>
+    <t>Zoe was friendly with everyone we passed.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="170" formatCode="hh:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,12 +330,20 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -156,34 +379,76 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="27">
     <dxf>
       <font>
         <strike val="0"/>
@@ -197,6 +462,70 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="170" formatCode="hh:mm:ss"/>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -212,48 +541,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -274,6 +561,7 @@
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -294,6 +582,7 @@
           <bgColor theme="3" tint="0.89999084444715716"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -308,6 +597,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -337,6 +627,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -351,20 +642,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -385,6 +663,7 @@
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -405,6 +684,19 @@
           <bgColor theme="3" tint="0.89999084444715716"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -416,14 +708,7 @@
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.89999084444715716"/>
-        </patternFill>
-      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -433,7 +718,7 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="0"/>
+        <color auto="1"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -444,8 +729,79 @@
           <bgColor theme="3" tint="0.89999084444715716"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.89999084444715716"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -462,55 +818,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B335E5B2-B7AD-4762-BF44-C42AA3E92FDB}" name="Table3" displayName="Table3" ref="A1:D6" totalsRowShown="0" headerRowDxfId="18">
-  <autoFilter ref="A1:D6" xr:uid="{B335E5B2-B7AD-4762-BF44-C42AA3E92FDB}"/>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B335E5B2-B7AD-4762-BF44-C42AA3E92FDB}" name="Table3" displayName="Table3" ref="A1:D12" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A1:D12" xr:uid="{B335E5B2-B7AD-4762-BF44-C42AA3E92FDB}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{80C424CD-BB3A-4298-8A33-4AB14830922C}" name="owner_id (PK)" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{868B76BA-5E64-4B57-B52D-01AE590DF59A}" name="owner_name"/>
-    <tableColumn id="3" xr3:uid="{AE0EA7D6-324F-4022-949D-B36D24E721B1}" name="phone_number"/>
-    <tableColumn id="4" xr3:uid="{4F399586-F23F-45A5-8233-15FA5DF37BD4}" name="email"/>
+    <tableColumn id="1" xr3:uid="{80C424CD-BB3A-4298-8A33-4AB14830922C}" name="owner_id " dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{868B76BA-5E64-4B57-B52D-01AE590DF59A}" name="owner_name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{AE0EA7D6-324F-4022-949D-B36D24E721B1}" name="phone_number" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{4F399586-F23F-45A5-8233-15FA5DF37BD4}" name="email" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{139D2D28-EFCC-49C1-A53E-E235293ADC54}" name="Table4" displayName="Table4" ref="A1:E6" totalsRowShown="0" headerRowDxfId="14">
-  <autoFilter ref="A1:E6" xr:uid="{139D2D28-EFCC-49C1-A53E-E235293ADC54}"/>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{139D2D28-EFCC-49C1-A53E-E235293ADC54}" name="Table4" displayName="Table4" ref="A1:E12" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A1:E12" xr:uid="{139D2D28-EFCC-49C1-A53E-E235293ADC54}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{C9C10A94-BBB3-43C0-968B-38EE22385182}" name="dog_id (PK)" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{C2714D09-162B-4C42-8B5D-7229997503D1}" name="owner_id (FK)" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{34445534-D457-4D7F-8C6A-4E28ED4FA7DC}" name="dog_name"/>
-    <tableColumn id="4" xr3:uid="{21D784F5-21C4-474F-9CF7-F7A6E1AA51BB}" name="breed"/>
-    <tableColumn id="5" xr3:uid="{8F63065B-72DA-4B93-80DB-A547E9CD3F3D}" name="age"/>
+    <tableColumn id="1" xr3:uid="{C9C10A94-BBB3-43C0-968B-38EE22385182}" name="dog_id " dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{C2714D09-162B-4C42-8B5D-7229997503D1}" name="owner_id " dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{34445534-D457-4D7F-8C6A-4E28ED4FA7DC}" name="dog_name" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{21D784F5-21C4-474F-9CF7-F7A6E1AA51BB}" name="breed" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{8F63065B-72DA-4B93-80DB-A547E9CD3F3D}" name="age" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6C4E8387-2403-4929-A86F-6A75BFD444B5}" name="Table5" displayName="Table5" ref="A1:E6" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:E6" xr:uid="{6C4E8387-2403-4929-A86F-6A75BFD444B5}"/>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6C4E8387-2403-4929-A86F-6A75BFD444B5}" name="Table5" displayName="Table5" ref="A1:E12" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:E12" xr:uid="{6C4E8387-2403-4929-A86F-6A75BFD444B5}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{06E20231-D9AB-41BF-BEF3-7116BE749241}" name="walk_id (PK)" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{6500AF60-F9C5-41CD-A427-7C0FC3A4BFA7}" name="dog_id (FK)" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{06E20231-D9AB-41BF-BEF3-7116BE749241}" name="walk_id " dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{6500AF60-F9C5-41CD-A427-7C0FC3A4BFA7}" name="dog_id " dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{933DB32B-8DA0-4A67-9221-9B8167AEB156}" name="walk_date" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{37A70DF2-1F30-43B3-A7C1-D69E5EB18474}" name="walk_duration" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{55C5F72B-9A3E-4203-9581-EA680786B0ED}" name="notes" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{37A70DF2-1F30-43B3-A7C1-D69E5EB18474}" name="walk_duration" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{55C5F72B-9A3E-4203-9581-EA680786B0ED}" name="notes" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{443EBC68-654A-40F9-9C0D-814B574680F5}" name="Table6" displayName="Table6" ref="A1:E7" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:E7" xr:uid="{443EBC68-654A-40F9-9C0D-814B574680F5}"/>
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{443EBC68-654A-40F9-9C0D-814B574680F5}" name="Table6" displayName="Table6" ref="A1:E12" totalsRowShown="0" headerRowDxfId="26" dataDxfId="3">
+  <autoFilter ref="A1:E12" xr:uid="{443EBC68-654A-40F9-9C0D-814B574680F5}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7BC331FF-D9AF-4646-A8C9-A1CC322052CB}" name="payment_id(PK)" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{435F1D1D-4E2F-4B4A-8EE2-1A1D5882592A}" name="owner_id (FK)" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{540F89FC-A9E4-4B8D-8383-1F058B36C275}" name="amount" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{C99CE62D-56AA-4875-885E-270D551F0932}" name="payment_method" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{1FAD9FA5-F486-47DD-BAA1-6CA888E42A56}" name="date_serviced" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{7BC331FF-D9AF-4646-A8C9-A1CC322052CB}" name="payment_id" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{435F1D1D-4E2F-4B4A-8EE2-1A1D5882592A}" name="owner_id " dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{540F89FC-A9E4-4B8D-8383-1F058B36C275}" name="amount" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{C99CE62D-56AA-4875-885E-270D551F0932}" name="payment_method" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{1FAD9FA5-F486-47DD-BAA1-6CA888E42A56}" name="date_serviced" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -833,79 +1189,408 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87CA01F9-40B5-46BE-BE52-FFD169ED4555}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.21875" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.77734375" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="4"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
+      <c r="B4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="4"/>
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>52</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{09109415-97CE-402B-97B6-05DEE302C854}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31BC9D7B-BD90-455D-9CF5-F52E79C3F8D6}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.77734375" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
         <v>8</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B9" s="3">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="2">
         <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -918,67 +1603,219 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEB45426-463C-4A45-B6CF-E0C9E34E5E52}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="71" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="17">
+        <v>101</v>
+      </c>
+      <c r="B2" s="18">
+        <v>1</v>
+      </c>
+      <c r="C2" s="10" t="d">
+        <v>2026-10-20T09:30:00.00000020954757600</v>
+      </c>
+      <c r="D2" s="11" t="d">
+        <v>00:45:00.000</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>102</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+      <c r="C3" s="10" t="d">
+        <v>2026-10-12T08:00:00.00000020954757600</v>
+      </c>
+      <c r="D3" s="9" t="d">
+        <v>00:29:59.99999999999990100</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>103</v>
+      </c>
+      <c r="B4" s="6">
+        <v>3</v>
+      </c>
+      <c r="C4" s="10" t="d">
+        <v>2026-10-12T10:15:00.00000020954757600</v>
+      </c>
+      <c r="D4" s="9" t="d">
+        <v>00:59:59.99999999999980200</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
+        <v>104</v>
+      </c>
+      <c r="B5" s="6">
+        <v>4</v>
+      </c>
+      <c r="C5" s="10" t="d">
+        <v>2026-10-13T09:00:00.000</v>
+      </c>
+      <c r="D5" s="9" t="d">
+        <v>00:29:59.99999999999990100</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>105</v>
+      </c>
+      <c r="B6" s="6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="10" t="d">
+        <v>2026-10-13T12:30:00.00000020954757600</v>
+      </c>
+      <c r="D6" s="9" t="d">
+        <v>00:19:59.99999999999993400</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
+        <v>106</v>
+      </c>
+      <c r="B7" s="6">
+        <v>6</v>
+      </c>
+      <c r="C7" s="10" t="d">
+        <v>2026-10-14T08:45:00.00000020954757600</v>
+      </c>
+      <c r="D7" s="9" t="d">
+        <v>00:45:00.000</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>107</v>
+      </c>
+      <c r="B8" s="6">
+        <v>7</v>
+      </c>
+      <c r="C8" s="10" t="d">
+        <v>2026-10-14T15:59:59.99999979045242400</v>
+      </c>
+      <c r="D8" s="9" t="d">
+        <v>00:59:59.99999999999980200</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
+        <v>108</v>
+      </c>
+      <c r="B9" s="6">
+        <v>8</v>
+      </c>
+      <c r="C9" s="10" t="d">
+        <v>2026-10-15T07:30:00.000</v>
+      </c>
+      <c r="D9" s="9" t="d">
+        <v>00:45:00.000</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>109</v>
+      </c>
+      <c r="B10" s="6">
         <v>9</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="C10" s="10" t="d">
+        <v>2026-10-15T11:00:00.00000020954757600</v>
+      </c>
+      <c r="D10" s="9" t="d">
+        <v>00:25:00.00000000000006600</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>110</v>
+      </c>
+      <c r="B11" s="6">
         <v>10</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="C11" s="10" t="d">
+        <v>2026-10-16T17:29:59.99999979045242400</v>
+      </c>
+      <c r="D11" s="9" t="d">
+        <v>01:15:00.00000000000019800</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>111</v>
+      </c>
+      <c r="B12" s="6">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="C12" s="10" t="d">
+        <v>2026-10-16T12:59:59.99999979045242400</v>
+      </c>
+      <c r="D12" s="9" t="d">
+        <v>00:35:00.00000000000003300</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>87</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -990,74 +1827,219 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EBFFC7A-9C7A-4EF9-AAD2-CC05C51D2EE7}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" style="14" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" style="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>14</v>
+      <c r="A1" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="13">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="6">
+        <v>1</v>
+      </c>
+      <c r="C2" s="21">
+        <v>25</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="12" t="d">
+        <v>2026-10-20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="13">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+      <c r="C3" s="21">
+        <v>20</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="12" t="d">
+        <v>2026-10-12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="6">
+        <v>3</v>
+      </c>
+      <c r="C4" s="21">
+        <v>40</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="12" t="d">
+        <v>2026-10-12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="13">
+        <v>1004</v>
+      </c>
+      <c r="B5" s="6">
+        <v>4</v>
+      </c>
+      <c r="C5" s="21">
+        <v>20</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="12" t="d">
+        <v>2026-10-13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="13">
+        <v>1005</v>
+      </c>
+      <c r="B6" s="6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="21">
+        <v>15</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="12" t="d">
+        <v>2026-10-13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="13">
+        <v>1006</v>
+      </c>
+      <c r="B7" s="6">
+        <v>6</v>
+      </c>
+      <c r="C7" s="21">
+        <v>30</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="12" t="d">
+        <v>2026-10-14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="13">
+        <v>1007</v>
+      </c>
+      <c r="B8" s="6">
+        <v>7</v>
+      </c>
+      <c r="C8" s="21">
+        <v>40</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="12" t="d">
+        <v>2026-10-14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="13">
+        <v>1008</v>
+      </c>
+      <c r="B9" s="6">
         <v>8</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
+      <c r="C9" s="21">
+        <v>30</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="12" t="d">
+        <v>2026-10-15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="13">
+        <v>1009</v>
+      </c>
+      <c r="B10" s="6">
+        <v>9</v>
+      </c>
+      <c r="C10" s="21">
+        <v>20</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="12" t="d">
+        <v>2026-10-15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>1010</v>
+      </c>
+      <c r="B11" s="6">
+        <v>10</v>
+      </c>
+      <c r="C11" s="21">
+        <v>50</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="12" t="d">
+        <v>2026-10-16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>1011</v>
+      </c>
+      <c r="B12" s="6">
+        <v>11</v>
+      </c>
+      <c r="C12" s="21">
+        <v>25</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="12" t="d">
+        <v>2026-10-16</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>